<commit_message>
Site updated: 2021-01-17 19:45:53
</commit_message>
<xml_diff>
--- a/download/最新陸股分析估值報告.xlsx
+++ b/download/最新陸股分析估值報告.xlsx
@@ -9,11 +9,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
   </bookViews>
   <sheets>
-    <sheet name="【台灣】陸股ETF標的估值" sheetId="2" r:id="rId1"/>
-    <sheet name="【大陸】陸股ETF標的估值" sheetId="1" r:id="rId2"/>
+    <sheet name="【大陸】陸股ETF標的估值" sheetId="1" r:id="rId1"/>
+    <sheet name="【台灣】陸股ETF標的估值" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="105">
   <si>
     <t>行業</t>
   </si>
@@ -42,10 +42,6 @@
     <t>PB位置</t>
   </si>
   <si>
-    <t>Q2ROE</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>Yield</t>
   </si>
   <si>
@@ -68,22 +64,6 @@
   </si>
   <si>
     <t>ROE(%)</t>
-  </si>
-  <si>
-    <t>ETF名稱</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>代號</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>PE</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>標的指數</t>
-    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>上證50</t>
@@ -99,18 +79,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>元大寶滬深</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>0061</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>滬深300</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>滬深300</t>
   </si>
   <si>
@@ -124,18 +92,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>富邦上證</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>006205</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>上證180</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>中證500</t>
   </si>
   <si>
@@ -149,18 +105,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>元大上證50</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>006206</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>上證50</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>創業100</t>
   </si>
   <si>
@@ -174,18 +118,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>富邦深100</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>00639</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>深圳100</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>恒生指數</t>
   </si>
   <si>
@@ -196,18 +128,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>群益深證中小</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>00643</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>中小板</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>銀行</t>
   </si>
   <si>
@@ -221,14 +141,6 @@
     <t>富邦恒生國企</t>
   </si>
   <si>
-    <t>00700</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>-</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>恒生中國企業指數</t>
   </si>
   <si>
@@ -249,14 +161,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>元大標普500</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>00646</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -396,7 +300,72 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>11月中行業估值</t>
+    <t>Q3ROE</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>ETF名稱</t>
+  </si>
+  <si>
+    <t>代號</t>
+  </si>
+  <si>
+    <t>Q3ROE</t>
+  </si>
+  <si>
+    <t>標的指數</t>
+  </si>
+  <si>
+    <t>元大寶滬深</t>
+  </si>
+  <si>
+    <t>0061</t>
+  </si>
+  <si>
+    <t>富邦上證</t>
+  </si>
+  <si>
+    <t>006205</t>
+  </si>
+  <si>
+    <t>元大上證50</t>
+  </si>
+  <si>
+    <t>006206</t>
+  </si>
+  <si>
+    <t>富邦深100</t>
+  </si>
+  <si>
+    <t>00639</t>
+  </si>
+  <si>
+    <t>深圳100</t>
+  </si>
+  <si>
+    <t>群益深證中小</t>
+  </si>
+  <si>
+    <t>00643</t>
+  </si>
+  <si>
+    <t>中小板</t>
+  </si>
+  <si>
+    <t>00700</t>
+  </si>
+  <si>
+    <t>元大標普500</t>
+  </si>
+  <si>
+    <t>00646</t>
+  </si>
+  <si>
+    <t>1月中行業估值</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>-</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -668,512 +637,6 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>18415</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>80010</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="矩形 2"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5762625" y="1828800"/>
-          <a:ext cx="1189990" cy="251460"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="000000"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr rtlCol="0" anchor="ctr"/>
-        <a:lstStyle>
-          <a:defPPr>
-            <a:defRPr lang="zh-TW">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:defPPr>
-          <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl1pPr>
-          <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl2pPr>
-          <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl3pPr>
-          <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl4pPr>
-          <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl5pPr>
-          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl6pPr>
-          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl7pPr>
-          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl8pPr>
-          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl9pPr>
-        </a:lstStyle>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="900" dirty="0" smtClean="0">
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:latin typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
-              <a:ea typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
-            </a:rPr>
-            <a:t>隔壁表哥-輕鬆理財</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>333375</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>32385</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>8890</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>83820</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="矩形 2"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9677400" y="3861435"/>
-          <a:ext cx="1475740" cy="251460"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="000000"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr rtlCol="0" anchor="ctr"/>
-        <a:lstStyle>
-          <a:defPPr>
-            <a:defRPr lang="zh-TW">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:defPPr>
-          <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl1pPr>
-          <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl2pPr>
-          <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl3pPr>
-          <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl4pPr>
-          <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl5pPr>
-          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl6pPr>
-          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl7pPr>
-          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl8pPr>
-          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl9pPr>
-        </a:lstStyle>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1050" dirty="0" smtClean="0">
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:latin typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
-              <a:ea typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
-            </a:rPr>
-            <a:t>隔壁表哥-輕鬆理財</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>333375</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>31</xdr:col>
-      <xdr:colOff>8890</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>80010</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="矩形 2"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="15087600" y="4257675"/>
-          <a:ext cx="1475740" cy="251460"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="000000"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr rtlCol="0" anchor="ctr"/>
-        <a:lstStyle>
-          <a:defPPr>
-            <a:defRPr lang="zh-TW">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:defPPr>
-          <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl1pPr>
-          <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl2pPr>
-          <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl3pPr>
-          <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl4pPr>
-          <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl5pPr>
-          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl6pPr>
-          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl7pPr>
-          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl8pPr>
-          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr sz="1800" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="lt1"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:lvl9pPr>
-        </a:lstStyle>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1050" dirty="0" smtClean="0">
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:latin typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
-              <a:ea typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
-            </a:rPr>
-            <a:t>隔壁表哥-輕鬆理財</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>20</xdr:col>
       <xdr:colOff>333375</xdr:colOff>
       <xdr:row>17</xdr:row>
@@ -1493,6 +956,846 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="zh-CN" altLang="en-US" sz="1050" dirty="0" smtClean="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              <a:ea typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:rPr>
+            <a:t>隔壁表哥-輕鬆理財</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>32385</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>8890</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="矩形 2"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9677400" y="3432810"/>
+          <a:ext cx="1475740" cy="251460"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rtlCol="0" anchor="ctr"/>
+        <a:lstStyle>
+          <a:defPPr>
+            <a:defRPr lang="zh-TW">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:defPPr>
+          <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1050" dirty="0" smtClean="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              <a:ea typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:rPr>
+            <a:t>隔壁表哥-輕鬆理財</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>8890</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>80010</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="矩形 2"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15087600" y="3829050"/>
+          <a:ext cx="1475740" cy="251460"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rtlCol="0" anchor="ctr"/>
+        <a:lstStyle>
+          <a:defPPr>
+            <a:defRPr lang="zh-TW">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:defPPr>
+          <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1050" dirty="0" smtClean="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              <a:ea typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:rPr>
+            <a:t>隔壁表哥-輕鬆理財</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>32385</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>8890</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="矩形 2"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9725025" y="3432810"/>
+          <a:ext cx="1475740" cy="251460"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rtlCol="0" anchor="ctr"/>
+        <a:lstStyle>
+          <a:defPPr>
+            <a:defRPr lang="zh-TW">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:defPPr>
+          <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1050" dirty="0" smtClean="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              <a:ea typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:rPr>
+            <a:t>隔壁表哥-輕鬆理財</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>8890</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>80010</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="矩形 2"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15135225" y="3829050"/>
+          <a:ext cx="1475740" cy="251460"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rtlCol="0" anchor="ctr"/>
+        <a:lstStyle>
+          <a:defPPr>
+            <a:defRPr lang="zh-TW">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:defPPr>
+          <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1050" dirty="0" smtClean="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              <a:ea typeface="微软雅黑" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:rPr>
+            <a:t>隔壁表哥-輕鬆理財</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>18415</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>80010</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="矩形 2"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5838825" y="1828800"/>
+          <a:ext cx="1189990" cy="251460"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rtlCol="0" anchor="ctr"/>
+        <a:lstStyle>
+          <a:defPPr>
+            <a:defRPr lang="zh-TW">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:defPPr>
+          <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="900" dirty="0" smtClean="0">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -1772,485 +2075,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
-  <cols>
-    <col min="1" max="1" width="2.85546875" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="1"/>
-      <c r="B2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K2" s="1"/>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="1"/>
-      <c r="B3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="4">
-        <v>14.85</v>
-      </c>
-      <c r="E3" s="5">
-        <v>0.89880000000000004</v>
-      </c>
-      <c r="F3" s="4">
-        <v>1.59</v>
-      </c>
-      <c r="G3" s="5">
-        <v>0.57889999999999997</v>
-      </c>
-      <c r="H3" s="5">
-        <v>7.9600000000000004E-2</v>
-      </c>
-      <c r="I3" s="5">
-        <v>2.3300000000000001E-2</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="1"/>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="1"/>
-      <c r="B4" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D4" s="4">
-        <v>12.48</v>
-      </c>
-      <c r="E4" s="5">
-        <v>0.83220000000000005</v>
-      </c>
-      <c r="F4" s="4">
-        <v>1.3</v>
-      </c>
-      <c r="G4" s="5">
-        <v>0.30220000000000002</v>
-      </c>
-      <c r="H4" s="5">
-        <v>7.8E-2</v>
-      </c>
-      <c r="I4" s="5">
-        <v>2.8199999999999999E-2</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="K4" s="1"/>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="1"/>
-      <c r="B5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D5" s="4">
-        <v>11.62</v>
-      </c>
-      <c r="E5" s="5">
-        <v>0.85440000000000005</v>
-      </c>
-      <c r="F5" s="4">
-        <v>1.23</v>
-      </c>
-      <c r="G5" s="5">
-        <v>0.37709999999999999</v>
-      </c>
-      <c r="H5" s="5">
-        <v>7.4899999999999994E-2</v>
-      </c>
-      <c r="I5" s="5">
-        <v>3.0800000000000001E-2</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="K5" s="1"/>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="1"/>
-      <c r="B6" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="4">
-        <v>30.06</v>
-      </c>
-      <c r="E6" s="5">
-        <v>0.96130000000000004</v>
-      </c>
-      <c r="F6" s="4">
-        <v>4.1100000000000003</v>
-      </c>
-      <c r="G6" s="5">
-        <v>0.96750000000000003</v>
-      </c>
-      <c r="H6" s="5">
-        <v>9.8299999999999998E-2</v>
-      </c>
-      <c r="I6" s="5">
-        <v>1.06E-2</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="K6" s="1"/>
-    </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="1"/>
-      <c r="B7" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="4">
-        <v>35.96</v>
-      </c>
-      <c r="E7" s="5">
-        <v>0.84330000000000005</v>
-      </c>
-      <c r="F7" s="4">
-        <v>4.3600000000000003</v>
-      </c>
-      <c r="G7" s="5">
-        <v>0.69369999999999998</v>
-      </c>
-      <c r="H7" s="10">
-        <v>0.1048</v>
-      </c>
-      <c r="I7" s="5">
-        <v>8.3999999999999995E-3</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="K7" s="1"/>
-    </row>
-    <row r="8" spans="1:11">
-      <c r="A8" s="1"/>
-      <c r="B8" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="D8" s="4">
-        <v>11.59</v>
-      </c>
-      <c r="E8" s="5">
-        <v>0.93869999999999998</v>
-      </c>
-      <c r="F8" s="4">
-        <v>1.28</v>
-      </c>
-      <c r="G8" s="5">
-        <v>0.74409999999999998</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="I8" s="5">
-        <v>2.7799999999999998E-2</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="K8" s="1"/>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="1"/>
-      <c r="B9" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="D9" s="11">
-        <v>34.619999999999997</v>
-      </c>
-      <c r="E9" s="13">
-        <v>0.99639999999999995</v>
-      </c>
-      <c r="F9" s="11">
-        <v>3.84</v>
-      </c>
-      <c r="G9" s="13">
-        <v>0.99319999999999997</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="I9" s="13">
-        <v>1.5599999999999999E-2</v>
-      </c>
-      <c r="J9" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="K9" s="1"/>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-    </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="E3:E7">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G7">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H7">
-    <cfRule type="dataBar" priority="9">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFB628"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{16196E30-827E-4933-B837-C3496A41E6E2}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E8">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G8">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H8">
-    <cfRule type="dataBar" priority="5">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFB628"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4402D2D6-9822-4234-AC38-CE6669426211}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I8">
-    <cfRule type="dataBar" priority="6">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF008AEF"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{817E3484-488D-4C14-8F16-02CA61361451}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E9">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G9">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I9">
-    <cfRule type="dataBar" priority="10">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF008AEF"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{298DBD00-C8DD-4F04-95D0-EB96A1651133}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{16196E30-827E-4933-B837-C3496A41E6E2}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FFFFB628"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>H3:H7</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4402D2D6-9822-4234-AC38-CE6669426211}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FFFFB628"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>H8</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{817E3484-488D-4C14-8F16-02CA61361451}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF008AEF"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>I8</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{298DBD00-C8DD-4F04-95D0-EB96A1651133}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF008AEF"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>I3:I9</xm:sqref>
-        </x14:conditionalFormatting>
-      </x14:conditionalFormattings>
-    </ext>
-  </extLst>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:AR70"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
@@ -2265,7 +2089,9 @@
     <col min="9" max="9" width="13.85546875" style="1" hidden="1" customWidth="1"/>
     <col min="10" max="11" width="2.85546875" style="1" customWidth="1"/>
     <col min="12" max="12" width="11" style="1" customWidth="1"/>
-    <col min="13" max="15" width="9" style="1"/>
+    <col min="13" max="13" width="9" style="1"/>
+    <col min="14" max="14" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9" style="1"/>
     <col min="16" max="16" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="17" max="23" width="9" style="1"/>
     <col min="24" max="25" width="2.85546875" style="1" customWidth="1"/>
@@ -2285,7 +2111,7 @@
   <sheetData>
     <row r="2" spans="2:33">
       <c r="B2" s="25" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C2" s="26"/>
       <c r="D2" s="26"/>
@@ -2311,16 +2137,16 @@
         <v>4</v>
       </c>
       <c r="G3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>8</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>1</v>
@@ -2335,25 +2161,25 @@
         <v>4</v>
       </c>
       <c r="Q3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="R3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="S3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="T3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="U3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="U3" s="2" t="s">
+      <c r="V3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="V3" s="2" t="s">
+      <c r="W3" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="W3" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="Z3" s="2" t="s">
         <v>0</v>
@@ -2371,24 +2197,24 @@
         <v>4</v>
       </c>
       <c r="AE3" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AF3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AG3" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="AG3" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="2:33">
       <c r="B4" s="4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C4" s="4">
-        <v>11.62</v>
+        <v>14.85</v>
       </c>
       <c r="D4" s="5">
-        <v>0.85440000000000005</v>
+        <v>0.99880000000000002</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="5"/>
@@ -2396,37 +2222,37 @@
         <v>7.4899999999999994E-2</v>
       </c>
       <c r="H4" s="5">
-        <v>3.0800000000000001E-2</v>
+        <v>2.4500000000000001E-2</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="M4" s="4">
-        <v>7.04</v>
+        <v>6.85</v>
       </c>
       <c r="N4" s="5">
-        <v>0.21959999999999999</v>
+        <v>0.18129999999999999</v>
       </c>
       <c r="O4" s="7">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="P4" s="8">
-        <v>1.44E-2</v>
+        <v>9.4999999999999998E-3</v>
       </c>
       <c r="Q4" s="8">
         <v>7.9100000000000004E-2</v>
       </c>
       <c r="R4" s="8">
-        <v>5.1799999999999999E-2</v>
+        <v>5.2400000000000002E-2</v>
       </c>
       <c r="S4" s="4">
         <v>510880</v>
       </c>
       <c r="T4" s="9" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="U4" s="10">
         <v>5.0000000000000001E-3</v>
@@ -2439,39 +2265,39 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z4" s="4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="AA4" s="4">
-        <v>11.62</v>
+        <v>14.85</v>
       </c>
       <c r="AB4" s="5">
-        <v>0.85440000000000005</v>
+        <v>0.99880000000000002</v>
       </c>
       <c r="AC4" s="4">
-        <v>1.23</v>
+        <v>1.6</v>
       </c>
       <c r="AD4" s="5">
-        <v>0.37709999999999999</v>
+        <v>0.79769999999999996</v>
       </c>
       <c r="AE4" s="5">
         <v>7.4899999999999994E-2</v>
       </c>
       <c r="AF4" s="5">
-        <v>3.0800000000000001E-2</v>
+        <v>2.4500000000000001E-2</v>
       </c>
       <c r="AG4" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="2:33">
       <c r="B5" s="4" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C5" s="4">
-        <v>14.85</v>
+        <v>16.850000000000001</v>
       </c>
       <c r="D5" s="5">
-        <v>0.89880000000000004</v>
+        <v>0.98599999999999999</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="5"/>
@@ -2479,35 +2305,37 @@
         <v>7.9600000000000004E-2</v>
       </c>
       <c r="H5" s="5">
-        <v>2.3300000000000001E-2</v>
+        <v>2.0299999999999999E-2</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="M5" s="4">
-        <v>10.6</v>
+        <v>14.22</v>
       </c>
       <c r="N5" s="5">
-        <v>0.83179999999999998</v>
+        <v>0.99760000000000004</v>
       </c>
       <c r="O5" s="4">
-        <v>1.01</v>
+        <v>1.4</v>
       </c>
       <c r="P5" s="5">
-        <v>0.19900000000000001</v>
-      </c>
-      <c r="Q5" s="5"/>
+        <v>0.98709999999999998</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>104</v>
+      </c>
       <c r="R5" s="5">
-        <v>2.4E-2</v>
+        <v>1.7100000000000001E-2</v>
       </c>
       <c r="S5" s="4">
         <v>501050</v>
       </c>
       <c r="T5" s="9" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="U5" s="10">
         <v>5.0000000000000001E-3</v>
@@ -2520,39 +2348,39 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z5" s="4" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="AA5" s="4">
-        <v>14.85</v>
+        <v>16.850000000000001</v>
       </c>
       <c r="AB5" s="5">
-        <v>0.89880000000000004</v>
+        <v>0.98599999999999999</v>
       </c>
       <c r="AC5" s="4">
-        <v>1.59</v>
+        <v>1.83</v>
       </c>
       <c r="AD5" s="5">
-        <v>0.57889999999999997</v>
+        <v>0.83020000000000005</v>
       </c>
       <c r="AE5" s="5">
         <v>7.9600000000000004E-2</v>
       </c>
       <c r="AF5" s="5">
-        <v>2.3300000000000001E-2</v>
+        <v>2.0299999999999999E-2</v>
       </c>
       <c r="AG5" s="6" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="2:33">
       <c r="B6" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="C6" s="4">
-        <v>29.02</v>
+        <v>28.46</v>
       </c>
       <c r="D6" s="5">
-        <v>0.39839999999999998</v>
+        <v>0.3664</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="5"/>
@@ -2560,37 +2388,37 @@
         <v>5.3499999999999999E-2</v>
       </c>
       <c r="H6" s="5">
-        <v>1.2200000000000001E-2</v>
+        <v>1.26E-2</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="M6" s="4">
-        <v>10.28</v>
+        <v>11.04</v>
       </c>
       <c r="N6" s="5">
-        <v>0.79649999999999999</v>
+        <v>0.89759999999999995</v>
       </c>
       <c r="O6" s="4">
-        <v>1.1100000000000001</v>
+        <v>1.19</v>
       </c>
       <c r="P6" s="5">
-        <v>0.19239999999999999</v>
+        <v>0.44119999999999998</v>
       </c>
       <c r="Q6" s="5">
         <v>7.85E-2</v>
       </c>
       <c r="R6" s="5">
-        <v>3.49E-2</v>
+        <v>3.2500000000000001E-2</v>
       </c>
       <c r="S6" s="4">
         <v>160716</v>
       </c>
       <c r="T6" s="9" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="U6" s="10">
         <v>0.01</v>
@@ -2603,77 +2431,77 @@
         <v>1.18E-2</v>
       </c>
       <c r="Z6" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="AA6" s="4">
-        <v>29.02</v>
+        <v>28.46</v>
       </c>
       <c r="AB6" s="5">
-        <v>0.39839999999999998</v>
+        <v>0.3664</v>
       </c>
       <c r="AC6" s="4">
-        <v>2.08</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="AD6" s="5">
-        <v>0.21590000000000001</v>
+        <v>0.21959999999999999</v>
       </c>
       <c r="AE6" s="5">
         <v>5.3499999999999999E-2</v>
       </c>
       <c r="AF6" s="5">
-        <v>1.2200000000000001E-2</v>
+        <v>1.26E-2</v>
       </c>
       <c r="AG6" s="6" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="2:33">
       <c r="B7" s="4" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="C7" s="4">
-        <v>30.06</v>
+        <v>67</v>
       </c>
       <c r="D7" s="5">
-        <v>0.96130000000000004</v>
+        <v>0.88529999999999998</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5">
-        <v>9.8299999999999998E-2</v>
+        <v>0.108</v>
       </c>
       <c r="H7" s="5">
-        <v>1.06E-2</v>
+        <v>3.5999999999999999E-3</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="M7" s="4">
-        <v>8.01</v>
+        <v>7.84</v>
       </c>
       <c r="N7" s="5">
-        <v>0.34420000000000001</v>
+        <v>0.2989</v>
       </c>
       <c r="O7" s="4">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="P7" s="5">
-        <v>4.0300000000000002E-2</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="Q7" s="5">
         <v>8.2699999999999996E-2</v>
       </c>
       <c r="R7" s="5">
-        <v>4.5199999999999997E-2</v>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="S7" s="4">
         <v>161907</v>
       </c>
       <c r="T7" s="9" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="U7" s="10">
         <v>7.4999999999999997E-3</v>
@@ -2686,75 +2514,77 @@
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="Z7" s="4" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="AA7" s="4">
-        <v>30.06</v>
+        <v>67</v>
       </c>
       <c r="AB7" s="5">
-        <v>0.96130000000000004</v>
+        <v>0.88529999999999998</v>
       </c>
       <c r="AC7" s="4">
-        <v>4.1100000000000003</v>
+        <v>8.7200000000000006</v>
       </c>
       <c r="AD7" s="5">
-        <v>0.96750000000000003</v>
+        <v>0.93340000000000001</v>
       </c>
       <c r="AE7" s="5">
-        <v>9.8299999999999998E-2</v>
+        <v>0.108</v>
       </c>
       <c r="AF7" s="5">
-        <v>1.06E-2</v>
+        <v>3.5999999999999999E-3</v>
       </c>
       <c r="AG7" s="6" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="2:33">
       <c r="B8" s="4" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="C8" s="4">
-        <v>14.17</v>
+        <v>15.8</v>
       </c>
       <c r="D8" s="5">
-        <v>0.98699999999999999</v>
+        <v>1</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="5"/>
-      <c r="G8" s="4"/>
+      <c r="G8" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="H8" s="5">
-        <v>2.6499999999999999E-2</v>
+        <v>2.2800000000000001E-2</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M8" s="4">
-        <v>11.62</v>
+        <v>14.85</v>
       </c>
       <c r="N8" s="5">
-        <v>0.85440000000000005</v>
+        <v>0.99880000000000002</v>
       </c>
       <c r="O8" s="4">
-        <v>1.23</v>
+        <v>1.6</v>
       </c>
       <c r="P8" s="5">
-        <v>0.37709999999999999</v>
+        <v>0.79769999999999996</v>
       </c>
       <c r="Q8" s="5">
         <v>7.4899999999999994E-2</v>
       </c>
       <c r="R8" s="5">
-        <v>3.0800000000000001E-2</v>
+        <v>2.4500000000000001E-2</v>
       </c>
       <c r="S8" s="4">
         <v>510050</v>
       </c>
       <c r="T8" s="9" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="U8" s="10">
         <v>5.0000000000000001E-3</v>
@@ -2767,37 +2597,39 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z8" s="4" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="AA8" s="4">
-        <v>14.17</v>
+        <v>15.8</v>
       </c>
       <c r="AB8" s="5">
-        <v>0.98699999999999999</v>
+        <v>1</v>
       </c>
       <c r="AC8" s="4">
-        <v>1.26</v>
+        <v>1.38</v>
       </c>
       <c r="AD8" s="5">
-        <v>0.45689999999999997</v>
-      </c>
-      <c r="AE8" s="4"/>
+        <v>0.73709999999999998</v>
+      </c>
+      <c r="AE8" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="AF8" s="5">
-        <v>2.6499999999999999E-2</v>
+        <v>2.2800000000000001E-2</v>
       </c>
       <c r="AG8" s="6" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="2:33">
       <c r="B9" s="4" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="C9" s="4">
-        <v>6.42</v>
+        <v>6.89</v>
       </c>
       <c r="D9" s="5">
-        <v>0.50580000000000003</v>
+        <v>0.73109999999999997</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="5"/>
@@ -2805,37 +2637,37 @@
         <v>8.43E-2</v>
       </c>
       <c r="H9" s="5">
-        <v>4.8500000000000001E-2</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="M9" s="4">
-        <v>14.85</v>
+        <v>16.850000000000001</v>
       </c>
       <c r="N9" s="5">
-        <v>0.89880000000000004</v>
+        <v>0.98599999999999999</v>
       </c>
       <c r="O9" s="4">
-        <v>1.59</v>
+        <v>1.83</v>
       </c>
       <c r="P9" s="5">
-        <v>0.57889999999999997</v>
+        <v>0.83020000000000005</v>
       </c>
       <c r="Q9" s="5">
         <v>7.9600000000000004E-2</v>
       </c>
       <c r="R9" s="5">
-        <v>2.3300000000000001E-2</v>
+        <v>2.0299999999999999E-2</v>
       </c>
       <c r="S9" s="4">
         <v>510300</v>
       </c>
       <c r="T9" s="9" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="U9" s="10">
         <v>5.0000000000000001E-3</v>
@@ -2848,39 +2680,39 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z9" s="4" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="AA9" s="4">
-        <v>6.42</v>
+        <v>6.89</v>
       </c>
       <c r="AB9" s="5">
-        <v>0.50580000000000003</v>
+        <v>0.73109999999999997</v>
       </c>
       <c r="AC9" s="4">
-        <v>0.71</v>
+        <v>0.76</v>
       </c>
       <c r="AD9" s="5">
-        <v>1.32E-2</v>
+        <v>7.9799999999999996E-2</v>
       </c>
       <c r="AE9" s="5">
         <v>8.43E-2</v>
       </c>
       <c r="AF9" s="5">
-        <v>4.8500000000000001E-2</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="AG9" s="6" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="2:33">
       <c r="B10" s="4" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="C10" s="4">
-        <v>23.98</v>
+        <v>25.71</v>
       </c>
       <c r="D10" s="5">
-        <v>0.3856</v>
+        <v>0.49859999999999999</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="5"/>
@@ -2888,37 +2720,37 @@
         <v>6.9500000000000006E-2</v>
       </c>
       <c r="H10" s="5">
-        <v>1.1299999999999999E-2</v>
+        <v>1.01E-2</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="M10" s="4">
-        <v>35.32</v>
+        <v>41.66</v>
       </c>
       <c r="N10" s="5">
-        <v>0.86760000000000004</v>
+        <v>0.97940000000000005</v>
       </c>
       <c r="O10" s="4">
-        <v>8.4</v>
+        <v>9.6199999999999992</v>
       </c>
       <c r="P10" s="5">
-        <v>0.96499999999999997</v>
+        <v>0.99339999999999995</v>
       </c>
       <c r="Q10" s="5">
         <v>0.2009</v>
       </c>
       <c r="R10" s="5">
-        <v>1.11E-2</v>
+        <v>9.7999999999999997E-3</v>
       </c>
       <c r="S10" s="4">
         <v>159928</v>
       </c>
       <c r="T10" s="9" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="U10" s="10">
         <v>5.0000000000000001E-3</v>
@@ -2931,39 +2763,39 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z10" s="4" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="AA10" s="4">
-        <v>23.98</v>
+        <v>25.71</v>
       </c>
       <c r="AB10" s="5">
-        <v>0.3856</v>
+        <v>0.49859999999999999</v>
       </c>
       <c r="AC10" s="4">
-        <v>1.92</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="AD10" s="5">
-        <v>0.56179999999999997</v>
+        <v>0.72150000000000003</v>
       </c>
       <c r="AE10" s="5">
         <v>6.9500000000000006E-2</v>
       </c>
       <c r="AF10" s="5">
-        <v>1.1299999999999999E-2</v>
+        <v>1.01E-2</v>
       </c>
       <c r="AG10" s="6" t="s">
-        <v>63</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="2:33">
       <c r="B11" s="4" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="C11" s="4">
-        <v>6.82</v>
+        <v>6.59</v>
       </c>
       <c r="D11" s="5">
-        <v>1.8100000000000002E-2</v>
+        <v>8.6E-3</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="5"/>
@@ -2971,37 +2803,37 @@
         <v>8.0100000000000005E-2</v>
       </c>
       <c r="H11" s="5">
-        <v>4.53E-2</v>
+        <v>4.6899999999999997E-2</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="M11" s="4">
-        <v>63.66</v>
+        <v>67</v>
       </c>
       <c r="N11" s="5">
-        <v>0.82399999999999995</v>
+        <v>0.88529999999999998</v>
       </c>
       <c r="O11" s="4">
-        <v>7.47</v>
+        <v>8.7200000000000006</v>
       </c>
       <c r="P11" s="5">
-        <v>0.88280000000000003</v>
+        <v>0.93340000000000001</v>
       </c>
       <c r="Q11" s="5">
         <v>0.108</v>
       </c>
       <c r="R11" s="5">
-        <v>4.5999999999999999E-3</v>
+        <v>3.5999999999999999E-3</v>
       </c>
       <c r="S11" s="4">
         <v>159915</v>
       </c>
       <c r="T11" s="9" t="s">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="U11" s="10">
         <v>5.0000000000000001E-3</v>
@@ -3014,39 +2846,39 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z11" s="4" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="AA11" s="4">
-        <v>6.82</v>
+        <v>6.59</v>
       </c>
       <c r="AB11" s="5">
-        <v>1.8100000000000002E-2</v>
+        <v>8.6E-3</v>
       </c>
       <c r="AC11" s="4">
-        <v>1.33</v>
+        <v>1.29</v>
       </c>
       <c r="AD11" s="5">
-        <v>2.6700000000000002E-2</v>
+        <v>9.9000000000000008E-3</v>
       </c>
       <c r="AE11" s="5">
         <v>8.0100000000000005E-2</v>
       </c>
       <c r="AF11" s="5">
-        <v>4.53E-2</v>
+        <v>4.6899999999999997E-2</v>
       </c>
       <c r="AG11" s="6" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="2:33">
       <c r="B12" s="4" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="C12" s="4">
-        <v>7.5</v>
+        <v>7.29</v>
       </c>
       <c r="D12" s="5">
-        <v>8.3000000000000001E-3</v>
+        <v>1.61E-2</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="5"/>
@@ -3054,37 +2886,37 @@
         <v>6.2899999999999998E-2</v>
       </c>
       <c r="H12" s="5">
-        <v>2.53E-2</v>
+        <v>2.5600000000000001E-2</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="M12" s="4">
-        <v>12.48</v>
+        <v>14.3</v>
       </c>
       <c r="N12" s="5">
-        <v>0.83220000000000005</v>
+        <v>0.96419999999999995</v>
       </c>
       <c r="O12" s="4">
-        <v>1.3</v>
+        <v>1.49</v>
       </c>
       <c r="P12" s="5">
-        <v>0.30220000000000002</v>
+        <v>0.67310000000000003</v>
       </c>
       <c r="Q12" s="5">
         <v>7.8E-2</v>
       </c>
       <c r="R12" s="5">
-        <v>2.8199999999999999E-2</v>
+        <v>2.46E-2</v>
       </c>
       <c r="S12" s="4">
         <v>510180</v>
       </c>
       <c r="T12" s="9" t="s">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="U12" s="10">
         <v>5.0000000000000001E-3</v>
@@ -3097,39 +2929,39 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z12" s="4" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="AA12" s="4">
-        <v>7.5</v>
+        <v>7.29</v>
       </c>
       <c r="AB12" s="5">
-        <v>8.3000000000000001E-3</v>
+        <v>1.61E-2</v>
       </c>
       <c r="AC12" s="4">
         <v>0.82</v>
       </c>
       <c r="AD12" s="5">
-        <v>1.9699999999999999E-2</v>
+        <v>3.3000000000000002E-2</v>
       </c>
       <c r="AE12" s="5">
         <v>6.2899999999999998E-2</v>
       </c>
       <c r="AF12" s="5">
-        <v>2.53E-2</v>
+        <v>2.5600000000000001E-2</v>
       </c>
       <c r="AG12" s="6" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="2:33">
       <c r="B13" s="4" t="s">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="C13" s="4">
-        <v>48.41</v>
+        <v>59.43</v>
       </c>
       <c r="D13" s="5">
-        <v>0.94240000000000002</v>
+        <v>0.99670000000000003</v>
       </c>
       <c r="E13" s="4"/>
       <c r="F13" s="5"/>
@@ -3137,37 +2969,37 @@
         <v>0.1731</v>
       </c>
       <c r="H13" s="5">
-        <v>1.0200000000000001E-2</v>
+        <v>8.3000000000000001E-3</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>80</v>
+        <v>56</v>
       </c>
       <c r="M13" s="4">
-        <v>51.24</v>
+        <v>53.62</v>
       </c>
       <c r="N13" s="5">
-        <v>0.89490000000000003</v>
+        <v>0.90869999999999995</v>
       </c>
       <c r="O13" s="4">
-        <v>5.22</v>
+        <v>5.68</v>
       </c>
       <c r="P13" s="5">
-        <v>0.87809999999999999</v>
+        <v>0.91220000000000001</v>
       </c>
       <c r="Q13" s="5">
         <v>0.1057</v>
       </c>
       <c r="R13" s="5">
-        <v>6.7999999999999996E-3</v>
+        <v>6.1000000000000004E-3</v>
       </c>
       <c r="S13" s="4">
         <v>159938</v>
       </c>
       <c r="T13" s="9" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="U13" s="10">
         <v>5.0000000000000001E-3</v>
@@ -3180,39 +3012,39 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z13" s="4" t="s">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="AA13" s="4">
-        <v>48.41</v>
+        <v>59.43</v>
       </c>
       <c r="AB13" s="5">
-        <v>0.94240000000000002</v>
+        <v>0.99670000000000003</v>
       </c>
       <c r="AC13" s="4">
-        <v>10.08</v>
+        <v>12.82</v>
       </c>
       <c r="AD13" s="5">
-        <v>0.96630000000000005</v>
+        <v>0.99670000000000003</v>
       </c>
       <c r="AE13" s="5">
         <v>0.1731</v>
       </c>
       <c r="AF13" s="5">
-        <v>1.0200000000000001E-2</v>
+        <v>8.3000000000000001E-3</v>
       </c>
       <c r="AG13" s="6" t="s">
-        <v>82</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="2:33">
       <c r="B14" s="4" t="s">
-        <v>83</v>
+        <v>59</v>
       </c>
       <c r="C14" s="4">
-        <v>48.93</v>
+        <v>57.92</v>
       </c>
       <c r="D14" s="5">
-        <v>0.98919999999999997</v>
+        <v>0.99590000000000001</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="5"/>
@@ -3220,37 +3052,37 @@
         <v>0.1847</v>
       </c>
       <c r="H14" s="5">
-        <v>1.0500000000000001E-2</v>
+        <v>8.8999999999999999E-3</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="M14" s="4">
-        <v>30.06</v>
+        <v>35.21</v>
       </c>
       <c r="N14" s="5">
-        <v>0.96130000000000004</v>
+        <v>0.99139999999999995</v>
       </c>
       <c r="O14" s="4">
-        <v>4.1100000000000003</v>
+        <v>5.0599999999999996</v>
       </c>
       <c r="P14" s="5">
-        <v>0.96750000000000003</v>
+        <v>0.99670000000000003</v>
       </c>
       <c r="Q14" s="5">
         <v>9.8299999999999998E-2</v>
       </c>
       <c r="R14" s="5">
-        <v>1.06E-2</v>
+        <v>8.5000000000000006E-3</v>
       </c>
       <c r="S14" s="4">
         <v>159901</v>
       </c>
       <c r="T14" s="9" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
       <c r="U14" s="10">
         <v>5.0000000000000001E-3</v>
@@ -3263,39 +3095,39 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z14" s="4" t="s">
-        <v>83</v>
+        <v>59</v>
       </c>
       <c r="AA14" s="4">
-        <v>48.93</v>
+        <v>57.92</v>
       </c>
       <c r="AB14" s="5">
-        <v>0.98919999999999997</v>
+        <v>0.99590000000000001</v>
       </c>
       <c r="AC14" s="4">
-        <v>10.64</v>
+        <v>12.66</v>
       </c>
       <c r="AD14" s="5">
-        <v>0.96940000000000004</v>
+        <v>0.99590000000000001</v>
       </c>
       <c r="AE14" s="5">
         <v>0.1847</v>
       </c>
       <c r="AF14" s="5">
-        <v>1.0500000000000001E-2</v>
+        <v>8.8999999999999999E-3</v>
       </c>
       <c r="AG14" s="6" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="2:33">
       <c r="B15" s="4" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="C15" s="4">
-        <v>27.33</v>
+        <v>30.44</v>
       </c>
       <c r="D15" s="5">
-        <v>0.83889999999999998</v>
+        <v>0.94610000000000005</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="5"/>
@@ -3303,35 +3135,37 @@
         <v>0.1115</v>
       </c>
       <c r="H15" s="5">
-        <v>1.3899999999999999E-2</v>
+        <v>1.21E-2</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="M15" s="4">
-        <v>14.17</v>
+        <v>15.8</v>
       </c>
       <c r="N15" s="5">
-        <v>0.98699999999999999</v>
+        <v>1</v>
       </c>
       <c r="O15" s="4">
-        <v>1.26</v>
+        <v>1.38</v>
       </c>
       <c r="P15" s="5">
-        <v>0.45689999999999997</v>
-      </c>
-      <c r="Q15" s="4"/>
+        <v>0.73709999999999998</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>104</v>
+      </c>
       <c r="R15" s="5">
-        <v>2.6499999999999999E-2</v>
+        <v>2.2800000000000001E-2</v>
       </c>
       <c r="S15" s="4">
         <v>159920</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="U15" s="10">
         <v>6.4999999999999997E-3</v>
@@ -3344,39 +3178,39 @@
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="Z15" s="4" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="AA15" s="4">
-        <v>27.33</v>
+        <v>30.44</v>
       </c>
       <c r="AB15" s="5">
-        <v>0.83889999999999998</v>
+        <v>0.94610000000000005</v>
       </c>
       <c r="AC15" s="4">
-        <v>3.58</v>
+        <v>4.18</v>
       </c>
       <c r="AD15" s="5">
-        <v>0.83309999999999995</v>
+        <v>0.97270000000000001</v>
       </c>
       <c r="AE15" s="5">
         <v>0.1115</v>
       </c>
       <c r="AF15" s="5">
-        <v>1.3899999999999999E-2</v>
+        <v>1.21E-2</v>
       </c>
       <c r="AG15" s="6" t="s">
-        <v>91</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="2:33">
       <c r="B16" s="4" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="C16" s="4">
-        <v>58.92</v>
+        <v>73.58</v>
       </c>
       <c r="D16" s="5">
-        <v>0.17660000000000001</v>
+        <v>0.52029999999999998</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="5"/>
@@ -3384,37 +3218,37 @@
         <v>4.1599999999999998E-2</v>
       </c>
       <c r="H16" s="5">
-        <v>3.0999999999999999E-3</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="M16" s="4">
-        <v>42.46</v>
+        <v>44.03</v>
       </c>
       <c r="N16" s="5">
-        <v>0.99470000000000003</v>
+        <v>0.99739999999999995</v>
       </c>
       <c r="O16" s="4">
-        <v>2.78</v>
+        <v>2.97</v>
       </c>
       <c r="P16" s="5">
-        <v>0.66890000000000005</v>
+        <v>0.7883</v>
       </c>
       <c r="Q16" s="5">
         <v>5.8200000000000002E-2</v>
       </c>
       <c r="R16" s="5">
-        <v>1.35E-2</v>
+        <v>1.2699999999999999E-2</v>
       </c>
       <c r="S16" s="4">
         <v>159936</v>
       </c>
       <c r="T16" s="9" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="U16" s="10">
         <v>5.0000000000000001E-3</v>
@@ -3427,39 +3261,39 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z16" s="4" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="AA16" s="4">
-        <v>58.92</v>
+        <v>73.58</v>
       </c>
       <c r="AB16" s="5">
-        <v>0.17660000000000001</v>
+        <v>0.52029999999999998</v>
       </c>
       <c r="AC16" s="4">
-        <v>3.38</v>
+        <v>4.26</v>
       </c>
       <c r="AD16" s="5">
-        <v>0.55610000000000004</v>
+        <v>0.79879999999999995</v>
       </c>
       <c r="AE16" s="5">
         <v>4.1599999999999998E-2</v>
       </c>
       <c r="AF16" s="5">
-        <v>3.0999999999999999E-3</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="AG16" s="6" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="2:44">
       <c r="B17" s="4" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="C17" s="4">
-        <v>60.28</v>
+        <v>55.2</v>
       </c>
       <c r="D17" s="5">
-        <v>0.53369999999999995</v>
+        <v>0.44750000000000001</v>
       </c>
       <c r="E17" s="4"/>
       <c r="F17" s="5"/>
@@ -3467,37 +3301,37 @@
         <v>4.4699999999999997E-2</v>
       </c>
       <c r="H17" s="5">
-        <v>7.0000000000000001E-3</v>
+        <v>5.8999999999999999E-3</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="M17" s="11">
-        <v>29.02</v>
+        <v>28.46</v>
       </c>
       <c r="N17" s="13">
-        <v>0.39839999999999998</v>
+        <v>0.3664</v>
       </c>
       <c r="O17" s="11">
-        <v>2.08</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="P17" s="13">
-        <v>0.21590000000000001</v>
+        <v>0.21959999999999999</v>
       </c>
       <c r="Q17" s="13">
         <v>5.3499999999999999E-2</v>
       </c>
       <c r="R17" s="13">
-        <v>1.2200000000000001E-2</v>
+        <v>1.26E-2</v>
       </c>
       <c r="S17" s="11">
         <v>510500</v>
       </c>
       <c r="T17" s="12" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="U17" s="15">
         <v>5.0000000000000001E-3</v>
@@ -3510,28 +3344,28 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Z17" s="4" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="AA17" s="4">
-        <v>60.28</v>
+        <v>55.2</v>
       </c>
       <c r="AB17" s="5">
-        <v>0.53369999999999995</v>
+        <v>0.44750000000000001</v>
       </c>
       <c r="AC17" s="4">
-        <v>2.44</v>
+        <v>2.92</v>
       </c>
       <c r="AD17" s="5">
-        <v>0.48470000000000002</v>
+        <v>4.4699999999999997E-2</v>
       </c>
       <c r="AE17" s="5">
         <v>4.4699999999999997E-2</v>
       </c>
       <c r="AF17" s="5">
-        <v>7.0000000000000001E-3</v>
+        <v>5.8999999999999999E-3</v>
       </c>
       <c r="AG17" s="6" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="AJ17" s="16"/>
       <c r="AK17" s="16"/>
@@ -3545,13 +3379,13 @@
     </row>
     <row r="18" spans="2:44">
       <c r="B18" s="4" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="C18" s="4">
-        <v>59.18</v>
+        <v>64.84</v>
       </c>
       <c r="D18" s="5">
-        <v>0.41410000000000002</v>
+        <v>0.71779999999999999</v>
       </c>
       <c r="E18" s="4"/>
       <c r="F18" s="5"/>
@@ -3559,34 +3393,34 @@
         <v>0.1857</v>
       </c>
       <c r="H18" s="5">
-        <v>3.3E-3</v>
+        <v>2.8999999999999998E-3</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="Z18" s="4" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="AA18" s="4">
-        <v>59.18</v>
+        <v>64.84</v>
       </c>
       <c r="AB18" s="5">
-        <v>0.41410000000000002</v>
+        <v>0.71779999999999999</v>
       </c>
       <c r="AC18" s="4">
-        <v>9.56</v>
+        <v>11.35</v>
       </c>
       <c r="AD18" s="5">
-        <v>0.83779999999999999</v>
+        <v>0.93130000000000002</v>
       </c>
       <c r="AE18" s="5">
         <v>0.1857</v>
       </c>
       <c r="AF18" s="5">
-        <v>3.3E-3</v>
+        <v>2.8999999999999998E-3</v>
       </c>
       <c r="AG18" s="6" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="AJ18" s="16"/>
       <c r="AK18" s="16"/>
@@ -3600,13 +3434,13 @@
     </row>
     <row r="19" spans="2:44">
       <c r="B19" s="11" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="C19" s="11">
-        <v>48.96</v>
+        <v>54.4</v>
       </c>
       <c r="D19" s="13">
-        <v>0.77429999999999999</v>
+        <v>0.86839999999999995</v>
       </c>
       <c r="E19" s="11"/>
       <c r="F19" s="13"/>
@@ -3614,34 +3448,34 @@
         <v>7.8200000000000006E-2</v>
       </c>
       <c r="H19" s="13">
-        <v>5.8999999999999999E-3</v>
+        <v>5.3E-3</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="Z19" s="11" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="AA19" s="11">
-        <v>48.96</v>
+        <v>54.4</v>
       </c>
       <c r="AB19" s="13">
-        <v>0.77429999999999999</v>
+        <v>0.86839999999999995</v>
       </c>
       <c r="AC19" s="11">
-        <v>5.59</v>
+        <v>6.11</v>
       </c>
       <c r="AD19" s="13">
-        <v>0.85199999999999998</v>
+        <v>0.88449999999999995</v>
       </c>
       <c r="AE19" s="13">
         <v>7.8200000000000006E-2</v>
       </c>
       <c r="AF19" s="13">
-        <v>5.8999999999999999E-3</v>
+        <v>5.3E-3</v>
       </c>
       <c r="AG19" s="14" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="AJ19" s="16"/>
       <c r="AK19" s="16"/>
@@ -3733,7 +3567,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q8">
-    <cfRule type="dataBar" priority="20">
+    <cfRule type="dataBar" priority="19">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3741,27 +3575,13 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AD8AC959-0758-4BDB-9620-B3B25C9974DB}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R8">
-    <cfRule type="dataBar" priority="19">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF008AEF"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{351DC175-DD0F-479B-9957-4E79CAE05C7B}</x14:id>
+          <x14:id>{577FC6D6-9ECF-4DBE-8DAB-E057BDC4601C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N9">
-    <cfRule type="colorScale" priority="9">
+    <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3771,7 +3591,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P9">
-    <cfRule type="colorScale" priority="10">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3789,21 +3609,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7B960039-2032-469E-BA12-B03F32CA2CD6}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R9">
-    <cfRule type="dataBar" priority="11">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF008AEF"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7E455650-DCF8-44A6-8ECD-D30663EC8478}</x14:id>
+          <x14:id>{7C0D39EC-529F-41B8-ABA1-FF6CCDC42D70}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3837,7 +3643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EFA8E26F-218F-4425-B49B-9C42E4E1CF89}</x14:id>
+          <x14:id>{C7F8AD1D-D33D-4A56-A147-92A502257C16}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3851,12 +3657,22 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AA8D1622-1DFC-4118-BCFA-3F75FE591F07}</x14:id>
+          <x14:id>{9F2977FE-254A-4E12-A153-4C5E355C6CCF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N17">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P17">
     <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
@@ -3866,8 +3682,22 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P17">
-    <cfRule type="colorScale" priority="22">
+  <conditionalFormatting sqref="R17">
+    <cfRule type="dataBar" priority="22">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{482B90CF-0A7D-49F3-9F81-83F2C0DC94A4}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4:D21">
+    <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3876,21 +3706,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R17">
-    <cfRule type="dataBar" priority="23">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF008AEF"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{891CE3FF-B068-4329-8E91-3B7C2416F917}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D4:D21">
+  <conditionalFormatting sqref="F4:F21">
     <cfRule type="colorScale" priority="26">
       <colorScale>
         <cfvo type="min"/>
@@ -3900,18 +3716,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F4:F21">
-    <cfRule type="colorScale" priority="27">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="G4:G21">
-    <cfRule type="dataBar" priority="29">
+    <cfRule type="dataBar" priority="28">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3919,13 +3725,13 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{074D7A1F-BB7C-4A0B-A6D9-DAD0600BE621}</x14:id>
+          <x14:id>{D9A6E2E4-BB33-40F5-9AAE-467163C370F2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H21">
-    <cfRule type="dataBar" priority="28">
+    <cfRule type="dataBar" priority="27">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3933,13 +3739,13 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{24819C6A-4952-411F-A9CF-16F5459322F6}</x14:id>
+          <x14:id>{E54C89B9-06DD-458C-AFD1-CBE1DEE127DD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N4:N17">
-    <cfRule type="colorScale" priority="7">
+    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3949,7 +3755,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P4:P17">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3959,7 +3765,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W4:W17">
-    <cfRule type="dataBar" priority="30">
+    <cfRule type="dataBar" priority="29">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3967,13 +3773,13 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{075B5C8B-082B-4C65-B5E1-949E85B4E77D}</x14:id>
+          <x14:id>{8B9736D8-8F10-41E2-9FA8-736BB8985587}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N10:N14 N16 N4:N7">
-    <cfRule type="colorScale" priority="25">
+    <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3983,7 +3789,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P4:P7 P16 P10:P14">
-    <cfRule type="colorScale" priority="24">
+    <cfRule type="colorScale" priority="23">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3993,7 +3799,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q4:Q7 Q16 Q10:Q14">
-    <cfRule type="dataBar" priority="31">
+    <cfRule type="dataBar" priority="30">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4001,13 +3807,13 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4115F170-FE91-4ACC-BF8E-7A42BA64A5E8}</x14:id>
+          <x14:id>{23B9185C-3383-4EDB-8A38-73DE4A9055CA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R4:R7 R16 R10:R14">
-    <cfRule type="dataBar" priority="32">
+  <conditionalFormatting sqref="R10:R14 R16">
+    <cfRule type="dataBar" priority="31">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4015,13 +3821,13 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{328822F0-6976-4473-AEB0-5729B0D060B9}</x14:id>
+          <x14:id>{8CC3B3E2-FC25-449B-B3C4-20341209A5AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB4:AB19">
-    <cfRule type="colorScale" priority="3">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4031,7 +3837,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD4:AD19">
-    <cfRule type="colorScale" priority="4">
+    <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4041,7 +3847,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE4:AE19">
-    <cfRule type="dataBar" priority="6">
+    <cfRule type="dataBar" priority="7">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4049,13 +3855,13 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E712394D-4B6A-4264-B9BC-6EEAB00D7F17}</x14:id>
+          <x14:id>{D20FB20F-9809-4407-8D78-3D68E2FA3398}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF4:AF19">
-    <cfRule type="dataBar" priority="5">
+    <cfRule type="dataBar" priority="6">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4063,12 +3869,26 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D92EF317-C023-4CE8-8BA4-7C28732A4C4A}</x14:id>
+          <x14:id>{781E9A6D-052A-43A3-9FE1-494F3C4381B5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q17">
+    <cfRule type="dataBar" priority="3">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{2F58FC97-95C3-4202-A5F6-30949318EE08}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q4:Q17">
     <cfRule type="dataBar" priority="2">
       <dataBar>
         <cfvo type="min"/>
@@ -4077,26 +3897,22 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ED8DAC1E-58A3-4648-9FBE-10B331CC1BA4}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q4:Q17">
-    <cfRule type="dataBar" priority="1">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFB628"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C840F1FD-F3C4-4D3F-B9C4-87C072A8C914}</x14:id>
+          <x14:id>{20855EC5-EF8E-48A6-A9D0-1E3434DE273C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM17:AM19 AM22">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO17:AO19 AO22">
     <cfRule type="colorScale" priority="33">
       <colorScale>
         <cfvo type="min"/>
@@ -4106,18 +3922,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AO17:AO19 AO22">
-    <cfRule type="colorScale" priority="34">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="AP17:AP19 AP22">
-    <cfRule type="dataBar" priority="35">
+    <cfRule type="dataBar" priority="34">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4125,13 +3931,13 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BA0C3240-E439-4D42-BE7A-FEEBEA7E3BAB}</x14:id>
+          <x14:id>{BDDEF100-6B5A-40CD-B9AE-A5E68975C00A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AQ17:AQ19 AQ22">
-    <cfRule type="dataBar" priority="36">
+    <cfRule type="dataBar" priority="35">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4139,7 +3945,21 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{47A7F3BB-24D5-4516-AA70-739BD478B660}</x14:id>
+          <x14:id>{377000F7-9A0D-4E8E-B5F4-A806C3C1DD24}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R4:R17">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{BFAF4102-B00F-441F-93FC-77C2A8FCE52C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -4151,7 +3971,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AD8AC959-0758-4BDB-9620-B3B25C9974DB}">
+          <x14:cfRule type="dataBar" id="{577FC6D6-9ECF-4DBE-8DAB-E057BDC4601C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4164,20 +3984,7 @@
           <xm:sqref>Q8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{351DC175-DD0F-479B-9957-4E79CAE05C7B}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF008AEF"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>R8</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7B960039-2032-469E-BA12-B03F32CA2CD6}">
+          <x14:cfRule type="dataBar" id="{7C0D39EC-529F-41B8-ABA1-FF6CCDC42D70}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4190,20 +3997,7 @@
           <xm:sqref>Q9</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7E455650-DCF8-44A6-8ECD-D30663EC8478}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF008AEF"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>R9</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EFA8E26F-218F-4425-B49B-9C42E4E1CF89}">
+          <x14:cfRule type="dataBar" id="{C7F8AD1D-D33D-4A56-A147-92A502257C16}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4216,7 +4010,7 @@
           <xm:sqref>Q15</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AA8D1622-1DFC-4118-BCFA-3F75FE591F07}">
+          <x14:cfRule type="dataBar" id="{9F2977FE-254A-4E12-A153-4C5E355C6CCF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4229,7 +4023,7 @@
           <xm:sqref>R15</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{891CE3FF-B068-4329-8E91-3B7C2416F917}">
+          <x14:cfRule type="dataBar" id="{482B90CF-0A7D-49F3-9F81-83F2C0DC94A4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4242,7 +4036,7 @@
           <xm:sqref>R17</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{074D7A1F-BB7C-4A0B-A6D9-DAD0600BE621}">
+          <x14:cfRule type="dataBar" id="{D9A6E2E4-BB33-40F5-9AAE-467163C370F2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4255,7 +4049,7 @@
           <xm:sqref>G4:G21</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{24819C6A-4952-411F-A9CF-16F5459322F6}">
+          <x14:cfRule type="dataBar" id="{E54C89B9-06DD-458C-AFD1-CBE1DEE127DD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4268,7 +4062,7 @@
           <xm:sqref>H4:H21</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{075B5C8B-082B-4C65-B5E1-949E85B4E77D}">
+          <x14:cfRule type="dataBar" id="{8B9736D8-8F10-41E2-9FA8-736BB8985587}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4281,7 +4075,7 @@
           <xm:sqref>W4:W17</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4115F170-FE91-4ACC-BF8E-7A42BA64A5E8}">
+          <x14:cfRule type="dataBar" id="{23B9185C-3383-4EDB-8A38-73DE4A9055CA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4294,7 +4088,7 @@
           <xm:sqref>Q4:Q7 Q16 Q10:Q14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{328822F0-6976-4473-AEB0-5729B0D060B9}">
+          <x14:cfRule type="dataBar" id="{8CC3B3E2-FC25-449B-B3C4-20341209A5AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4304,10 +4098,10 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>R4:R7 R16 R10:R14</xm:sqref>
+          <xm:sqref>R10:R14 R16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E712394D-4B6A-4264-B9BC-6EEAB00D7F17}">
+          <x14:cfRule type="dataBar" id="{D20FB20F-9809-4407-8D78-3D68E2FA3398}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4320,7 +4114,7 @@
           <xm:sqref>AE4:AE19</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D92EF317-C023-4CE8-8BA4-7C28732A4C4A}">
+          <x14:cfRule type="dataBar" id="{781E9A6D-052A-43A3-9FE1-494F3C4381B5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4333,7 +4127,7 @@
           <xm:sqref>AF4:AF19</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ED8DAC1E-58A3-4648-9FBE-10B331CC1BA4}">
+          <x14:cfRule type="dataBar" id="{2F58FC97-95C3-4202-A5F6-30949318EE08}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4346,7 +4140,7 @@
           <xm:sqref>Q17</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C840F1FD-F3C4-4D3F-B9C4-87C072A8C914}">
+          <x14:cfRule type="dataBar" id="{20855EC5-EF8E-48A6-A9D0-1E3434DE273C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4359,7 +4153,7 @@
           <xm:sqref>Q4:Q17</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BA0C3240-E439-4D42-BE7A-FEEBEA7E3BAB}">
+          <x14:cfRule type="dataBar" id="{BDDEF100-6B5A-40CD-B9AE-A5E68975C00A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4372,7 +4166,7 @@
           <xm:sqref>AP17:AP19 AP22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{47A7F3BB-24D5-4516-AA70-739BD478B660}">
+          <x14:cfRule type="dataBar" id="{377000F7-9A0D-4E8E-B5F4-A806C3C1DD24}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -4384,6 +4178,500 @@
           </x14:cfRule>
           <xm:sqref>AQ17:AQ19 AQ22</xm:sqref>
         </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{BFAF4102-B00F-441F-93FC-77C2A8FCE52C}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>R4:R17</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="2.85546875" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="2.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="K2" s="1"/>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="1"/>
+      <c r="B3" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="4">
+        <v>16.850000000000001</v>
+      </c>
+      <c r="E3" s="5">
+        <v>0.98599999999999999</v>
+      </c>
+      <c r="F3" s="4">
+        <v>1.83</v>
+      </c>
+      <c r="G3" s="5">
+        <v>0.83020000000000005</v>
+      </c>
+      <c r="H3" s="5">
+        <v>7.9600000000000004E-2</v>
+      </c>
+      <c r="I3" s="5">
+        <v>2.0299999999999999E-2</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="1"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="1"/>
+      <c r="B4" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" s="4">
+        <v>14.3</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0.96419999999999995</v>
+      </c>
+      <c r="F4" s="4">
+        <v>1.49</v>
+      </c>
+      <c r="G4" s="5">
+        <v>0.67310000000000003</v>
+      </c>
+      <c r="H4" s="5">
+        <v>7.8E-2</v>
+      </c>
+      <c r="I4" s="5">
+        <v>2.46E-2</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K4" s="1"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="1"/>
+      <c r="B5" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5" s="4">
+        <v>14.85</v>
+      </c>
+      <c r="E5" s="5">
+        <v>0.99880000000000002</v>
+      </c>
+      <c r="F5" s="4">
+        <v>1.6</v>
+      </c>
+      <c r="G5" s="5">
+        <v>0.79769999999999996</v>
+      </c>
+      <c r="H5" s="5">
+        <v>7.4899999999999994E-2</v>
+      </c>
+      <c r="I5" s="5">
+        <v>2.4500000000000001E-2</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="1"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="1"/>
+      <c r="B6" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="4">
+        <v>67</v>
+      </c>
+      <c r="E6" s="5">
+        <v>0.88529999999999998</v>
+      </c>
+      <c r="F6" s="4">
+        <v>8.7200000000000006</v>
+      </c>
+      <c r="G6" s="5">
+        <v>0.93340000000000001</v>
+      </c>
+      <c r="H6" s="5">
+        <v>0.108</v>
+      </c>
+      <c r="I6" s="5">
+        <v>3.5999999999999999E-3</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="1"/>
+      <c r="B7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="4">
+        <v>36.909999999999997</v>
+      </c>
+      <c r="E7" s="5">
+        <v>0.89600000000000002</v>
+      </c>
+      <c r="F7" s="4">
+        <v>4.96</v>
+      </c>
+      <c r="G7" s="5">
+        <v>0.88729999999999998</v>
+      </c>
+      <c r="H7" s="10">
+        <v>0.1048</v>
+      </c>
+      <c r="I7" s="5">
+        <v>7.6E-3</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="K7" s="1"/>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="1"/>
+      <c r="B8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="D8" s="4">
+        <v>13.8</v>
+      </c>
+      <c r="E8" s="5">
+        <v>1</v>
+      </c>
+      <c r="F8" s="4">
+        <v>1.46</v>
+      </c>
+      <c r="G8" s="5">
+        <v>0.8992</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I8" s="5">
+        <v>2.2599999999999999E-2</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="K8" s="1"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="1"/>
+      <c r="B9" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" s="11">
+        <v>37.32</v>
+      </c>
+      <c r="E9" s="13">
+        <v>0.99760000000000004</v>
+      </c>
+      <c r="F9" s="11">
+        <v>4.2</v>
+      </c>
+      <c r="G9" s="13">
+        <v>0.99760000000000004</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="I9" s="13">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="K9" s="1"/>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="E3:E7">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3:G7">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3:H7">
+    <cfRule type="dataBar" priority="9">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{A430C4F9-1778-403D-84C5-641033C32010}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H8">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{2346D5CA-ABA4-4383-B71F-4F0EC5BAB0F2}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I8">
+    <cfRule type="dataBar" priority="6">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{B57F788D-2110-4DC6-A64C-BD61773D7413}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3:I9">
+    <cfRule type="dataBar" priority="10">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{A41E4E83-88F6-49EC-921D-C09B66CB1183}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{A430C4F9-1778-403D-84C5-641033C32010}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>H3:H7</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{2346D5CA-ABA4-4383-B71F-4F0EC5BAB0F2}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>H8</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{B57F788D-2110-4DC6-A64C-BD61773D7413}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>I8</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{A41E4E83-88F6-49EC-921D-C09B66CB1183}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>I3:I9</xm:sqref>
+        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>

</xml_diff>